<commit_message>
1811 S Bentley: year built 1964 per Filip
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/files/08-1811-s-bentley-ave.xlsx
+++ b/files/08-1811-s-bentley-ave.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\iniculete\LAAA-Deploys\onmarket\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3231C191-68DE-456D-96B0-81B4FEC64C4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F691ECDF-7756-4197-A014-F66C9B14961E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{EDF2B707-273B-4FA5-9354-3350A5F7182B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{42F1E642-2337-480A-A093-92B3B78A2CE0}"/>
   </bookViews>
   <sheets>
     <sheet name="Assumptions" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="145">
   <si>
     <t>LAAA UNDERWRITING BENCHMARKS (edit here; every deal tab reads these)</t>
   </si>
@@ -214,6 +214,9 @@
   </si>
   <si>
     <t>Year built</t>
+  </si>
+  <si>
+    <t>per Filip 9/17/2026 (LoopNet did not publish)</t>
   </si>
   <si>
     <t>Stories</t>
@@ -484,7 +487,7 @@
     <numFmt numFmtId="166" formatCode="0.00&quot;x&quot;"/>
     <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0;\(&quot;$&quot;#,##0\);&quot;-&quot;"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -531,6 +534,14 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFC00000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -621,7 +632,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -639,21 +650,22 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="167" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="3" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -686,7 +698,7 @@
         <xdr:cNvPr id="2" name="Image 1" descr="Picture">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{542EBF7E-8D4E-4E83-8C3B-C437E9B617E5}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E8AB4790-F825-493C-A2DD-FAFC02E9FED2}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -997,7 +1009,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC467143-0365-4747-B4F1-69805C3A98CC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{669D4272-E8F0-4D4B-A02A-ECC940FF2C00}">
   <dimension ref="A1:C40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1366,7 +1378,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0281AAAA-067A-4CEF-BE1C-4DF7B02328D7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{277CDC41-301A-466A-96A7-C64EDCF97A7D}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -1445,42 +1457,48 @@
       <c r="A11" t="s">
         <v>57</v>
       </c>
+      <c r="B11">
+        <v>1964</v>
+      </c>
+      <c r="C11" s="17" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B14" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B15" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B16" s="8">
         <v>5866611</v>
@@ -1488,38 +1506,38 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B17" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B18" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B19" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B21" s="14"/>
       <c r="C21" s="14"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B22" s="4">
         <v>6350000</v>
@@ -1527,7 +1545,7 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B23" s="8">
         <f>IFERROR(B22/B7,"")</f>
@@ -1536,32 +1554,32 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>76</v>
-      </c>
-      <c r="B24" s="17">
+        <v>77</v>
+      </c>
+      <c r="B24" s="18">
         <f>IFERROR(B22/B8,"")</f>
         <v>383.26895219700629</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>77</v>
-      </c>
-      <c r="B25" s="18">
+        <v>78</v>
+      </c>
+      <c r="B25" s="19">
         <v>5.6599999999999998E-2</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>78</v>
-      </c>
-      <c r="B26" s="19">
+        <v>79</v>
+      </c>
+      <c r="B26" s="20">
         <v>11.23</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="13" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B28" s="14"/>
       <c r="C28" s="14"/>
@@ -1570,137 +1588,137 @@
       <c r="F28" s="14"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A29" s="20" t="s">
-        <v>80</v>
-      </c>
-      <c r="B29" s="20" t="s">
+      <c r="A29" s="21" t="s">
         <v>81</v>
       </c>
-      <c r="C29" s="20" t="s">
+      <c r="B29" s="21" t="s">
         <v>82</v>
       </c>
-      <c r="D29" s="20" t="s">
+      <c r="C29" s="21" t="s">
         <v>83</v>
       </c>
-      <c r="E29" s="20" t="s">
+      <c r="D29" s="21" t="s">
         <v>84</v>
       </c>
-      <c r="F29" s="20" t="s">
+      <c r="E29" s="21" t="s">
         <v>85</v>
+      </c>
+      <c r="F29" s="21" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B30" s="15">
         <v>1</v>
       </c>
-      <c r="C30" s="21">
+      <c r="C30" s="22">
         <v>2900</v>
       </c>
-      <c r="D30" s="22">
+      <c r="D30" s="23">
         <f>B30*C30</f>
         <v>2900</v>
       </c>
-      <c r="E30" s="22">
+      <c r="E30" s="23">
         <f>D30*12</f>
         <v>34800</v>
       </c>
-      <c r="F30" s="23" t="s">
-        <v>87</v>
+      <c r="F30" s="24" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B31" s="15">
         <v>1</v>
       </c>
-      <c r="C31" s="21">
+      <c r="C31" s="22">
         <v>2648</v>
       </c>
-      <c r="D31" s="22">
+      <c r="D31" s="23">
         <f>B31*C31</f>
         <v>2648</v>
       </c>
-      <c r="E31" s="22">
+      <c r="E31" s="23">
         <f>D31*12</f>
         <v>31776</v>
       </c>
-      <c r="F31" s="23" t="s">
-        <v>87</v>
+      <c r="F31" s="24" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B32" s="15">
         <v>7</v>
       </c>
-      <c r="C32" s="21">
+      <c r="C32" s="22">
         <v>2699</v>
       </c>
-      <c r="D32" s="22">
+      <c r="D32" s="23">
         <f>B32*C32</f>
         <v>18893</v>
       </c>
-      <c r="E32" s="22">
+      <c r="E32" s="23">
         <f>D32*12</f>
         <v>226716</v>
       </c>
-      <c r="F32" s="23" t="s">
-        <v>87</v>
+      <c r="F32" s="24" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B33" s="15">
         <v>6</v>
       </c>
-      <c r="C33" s="21">
+      <c r="C33" s="22">
         <v>3780</v>
       </c>
-      <c r="D33" s="22">
+      <c r="D33" s="23">
         <f>B33*C33</f>
         <v>22680</v>
       </c>
-      <c r="E33" s="22">
+      <c r="E33" s="23">
         <f>D33*12</f>
         <v>272160</v>
       </c>
-      <c r="F33" s="23" t="s">
-        <v>87</v>
+      <c r="F33" s="24" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A34" s="24" t="s">
-        <v>91</v>
-      </c>
-      <c r="B34" s="25">
+      <c r="A34" s="25" t="s">
+        <v>92</v>
+      </c>
+      <c r="B34" s="26">
         <f>SUM(B30:B33)</f>
         <v>15</v>
       </c>
-      <c r="C34" s="26">
+      <c r="C34" s="27">
         <f>IFERROR(D34/B34,"")</f>
         <v>3141.4</v>
       </c>
-      <c r="D34" s="26">
+      <c r="D34" s="27">
         <f>SUM(D30:D33)</f>
         <v>47121</v>
       </c>
-      <c r="E34" s="26">
+      <c r="E34" s="27">
         <f>SUM(E30:E33)</f>
         <v>565452</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="13" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B36" s="14"/>
       <c r="C36" s="14"/>
@@ -1709,24 +1727,24 @@
       <c r="F36" s="14"/>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A37" s="27"/>
-      <c r="B37" s="27" t="s">
-        <v>93</v>
-      </c>
-      <c r="C37" s="27" t="s">
+      <c r="A37" s="28"/>
+      <c r="B37" s="28" t="s">
         <v>94</v>
       </c>
-      <c r="D37" s="27"/>
-      <c r="E37" s="27"/>
-      <c r="F37" s="27" t="s">
+      <c r="C37" s="28" t="s">
         <v>95</v>
+      </c>
+      <c r="D37" s="28"/>
+      <c r="E37" s="28"/>
+      <c r="F37" s="28" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>96</v>
-      </c>
-      <c r="B38" s="22">
+        <v>97</v>
+      </c>
+      <c r="B38" s="23">
         <v>565525</v>
       </c>
       <c r="C38" s="8">
@@ -1734,12 +1752,12 @@
         <v>565452</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B39" s="8">
         <v>2791</v>
@@ -1749,8 +1767,8 @@
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A40" s="24" t="s">
-        <v>99</v>
+      <c r="A40" s="25" t="s">
+        <v>100</v>
       </c>
       <c r="B40" s="8">
         <f>B38+B39</f>
@@ -1763,7 +1781,7 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B41" s="8">
         <f>-B38*0.03</f>
@@ -1774,25 +1792,25 @@
         <v>-16963.559999999998</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A42" s="24" t="s">
-        <v>102</v>
-      </c>
-      <c r="B42" s="26">
+      <c r="A42" s="25" t="s">
+        <v>103</v>
+      </c>
+      <c r="B42" s="27">
         <f>B40+B41</f>
         <v>551350.25</v>
       </c>
-      <c r="C42" s="26">
+      <c r="C42" s="27">
         <f>C40+C41</f>
         <v>551279.43999999994</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="13" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B44" s="14"/>
       <c r="C44" s="14"/>
@@ -1801,37 +1819,37 @@
       <c r="F44" s="14"/>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A45" s="27" t="s">
-        <v>104</v>
-      </c>
-      <c r="B45" s="27" t="s">
-        <v>93</v>
-      </c>
-      <c r="C45" s="27" t="s">
+      <c r="A45" s="28" t="s">
         <v>105</v>
       </c>
-      <c r="D45" s="27" t="s">
+      <c r="B45" s="28" t="s">
         <v>94</v>
       </c>
-      <c r="E45" s="27" t="s">
+      <c r="C45" s="28" t="s">
         <v>106</v>
       </c>
-      <c r="F45" s="27" t="s">
+      <c r="D45" s="28" t="s">
         <v>95</v>
+      </c>
+      <c r="E45" s="28" t="s">
+        <v>107</v>
+      </c>
+      <c r="F45" s="28" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>107</v>
-      </c>
-      <c r="B46" s="22">
+        <v>108</v>
+      </c>
+      <c r="B46" s="23">
         <v>75399</v>
       </c>
       <c r="C46" s="8">
         <f>B22*Assumptions!$B$15</f>
         <v>79375</v>
       </c>
-      <c r="D46" s="28">
+      <c r="D46" s="29">
         <f>C46</f>
         <v>79375</v>
       </c>
@@ -1840,21 +1858,21 @@
         <v>3976</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>109</v>
-      </c>
-      <c r="B47" s="22">
+        <v>110</v>
+      </c>
+      <c r="B47" s="23">
         <v>19527</v>
       </c>
       <c r="C47" s="8">
         <f>B7*Assumptions!$B$5+B8*Assumptions!$B$6</f>
         <v>19568</v>
       </c>
-      <c r="D47" s="28">
+      <c r="D47" s="29">
         <f t="shared" ref="D47:D53" si="1">IF(ISNUMBER(B47),MAX(B47,C47),C47)</f>
         <v>19568</v>
       </c>
@@ -1863,21 +1881,21 @@
         <v>41</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>111</v>
-      </c>
-      <c r="B48" s="22">
+        <v>112</v>
+      </c>
+      <c r="B48" s="23">
         <v>22054</v>
       </c>
       <c r="C48" s="8">
         <f>C42*Assumptions!$B$4</f>
         <v>27563.971999999998</v>
       </c>
-      <c r="D48" s="28">
+      <c r="D48" s="29">
         <f t="shared" si="1"/>
         <v>27563.971999999998</v>
       </c>
@@ -1886,21 +1904,21 @@
         <v>5509.9719999999979</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>113</v>
-      </c>
-      <c r="B49" s="22">
+        <v>114</v>
+      </c>
+      <c r="B49" s="23">
         <v>22500</v>
       </c>
       <c r="C49" s="8">
         <f>B7*Assumptions!$B$7</f>
         <v>18000</v>
       </c>
-      <c r="D49" s="28">
+      <c r="D49" s="29">
         <f t="shared" si="1"/>
         <v>22500</v>
       </c>
@@ -1909,21 +1927,21 @@
         <v>0</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>115</v>
-      </c>
-      <c r="B50" s="22">
+        <v>116</v>
+      </c>
+      <c r="B50" s="23">
         <v>28692</v>
       </c>
       <c r="C50" s="8">
         <f>B7*Assumptions!$B$9</f>
         <v>22500</v>
       </c>
-      <c r="D50" s="28">
+      <c r="D50" s="29">
         <f t="shared" si="1"/>
         <v>28692</v>
       </c>
@@ -1932,21 +1950,21 @@
         <v>0</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>117</v>
-      </c>
-      <c r="B51" s="22">
+        <v>118</v>
+      </c>
+      <c r="B51" s="23">
         <v>5646</v>
       </c>
       <c r="C51" s="8">
         <f>B7*Assumptions!$B$12</f>
         <v>6000</v>
       </c>
-      <c r="D51" s="28">
+      <c r="D51" s="29">
         <f t="shared" si="1"/>
         <v>6000</v>
       </c>
@@ -1955,21 +1973,21 @@
         <v>354</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>119</v>
-      </c>
-      <c r="B52" s="22">
+        <v>120</v>
+      </c>
+      <c r="B52" s="23">
         <v>12848</v>
       </c>
       <c r="C52" s="8">
         <f>B7*Assumptions!$B$13</f>
         <v>3750</v>
       </c>
-      <c r="D52" s="28">
+      <c r="D52" s="29">
         <f t="shared" si="1"/>
         <v>12848</v>
       </c>
@@ -1978,21 +1996,21 @@
         <v>0</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>121</v>
-      </c>
-      <c r="B53" s="22">
+        <v>122</v>
+      </c>
+      <c r="B53" s="23">
         <v>5250</v>
       </c>
       <c r="C53" s="8">
         <f>B7*Assumptions!$B$14</f>
         <v>4500</v>
       </c>
-      <c r="D53" s="28">
+      <c r="D53" s="29">
         <f t="shared" si="1"/>
         <v>5250</v>
       </c>
@@ -2001,36 +2019,36 @@
         <v>0</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A54" s="24" t="s">
-        <v>122</v>
-      </c>
-      <c r="B54" s="26">
+      <c r="A54" s="25" t="s">
+        <v>123</v>
+      </c>
+      <c r="B54" s="27">
         <f>SUM(B46:B53)</f>
         <v>191916</v>
       </c>
-      <c r="C54" s="26">
+      <c r="C54" s="27">
         <f>SUM(C46:C53)</f>
         <v>181256.97200000001</v>
       </c>
-      <c r="D54" s="26">
+      <c r="D54" s="27">
         <f>SUM(D46:D53)</f>
         <v>201796.97200000001</v>
       </c>
-      <c r="E54" s="26">
+      <c r="E54" s="27">
         <f t="shared" si="0"/>
         <v>9880.9720000000088</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B55" s="8">
         <f>IFERROR(B54/B7,"")</f>
@@ -2047,33 +2065,33 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>125</v>
-      </c>
-      <c r="B56" s="18">
+        <v>126</v>
+      </c>
+      <c r="B56" s="19">
         <f>IFERROR(B54/B42,"")</f>
         <v>0.34808363649059743</v>
       </c>
-      <c r="C56" s="18">
+      <c r="C56" s="19">
         <f>IFERROR(C54/C42,"")</f>
         <v>0.32879327406079217</v>
       </c>
-      <c r="D56" s="18">
+      <c r="D56" s="19">
         <f>IF(C38&gt;0,IFERROR(D54/C42,""),"")</f>
         <v>0.36605205519726985</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A57" s="24" t="s">
-        <v>126</v>
-      </c>
-      <c r="B57" s="29" t="str">
+      <c r="A57" s="25" t="s">
+        <v>127</v>
+      </c>
+      <c r="B57" s="30" t="str">
         <f>IF(ISNUMBER(B54),IF(D54&gt;B54*(1+Assumptions!$B$24),"OM EXPENSES LIGHT","OM expenses reasonable"),"OM expenses not published")</f>
         <v>OM EXPENSES LIGHT</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="13" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B59" s="14"/>
       <c r="C59" s="14"/>
@@ -2082,67 +2100,67 @@
       <c r="F59" s="14"/>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A60" s="27"/>
-      <c r="B60" s="27" t="s">
-        <v>93</v>
-      </c>
-      <c r="C60" s="27" t="s">
+      <c r="A60" s="28"/>
+      <c r="B60" s="28" t="s">
         <v>94</v>
       </c>
-      <c r="D60" s="27"/>
-      <c r="E60" s="27"/>
-      <c r="F60" s="27" t="s">
+      <c r="C60" s="28" t="s">
         <v>95</v>
       </c>
+      <c r="D60" s="28"/>
+      <c r="E60" s="28"/>
+      <c r="F60" s="28" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A61" s="24" t="s">
-        <v>128</v>
-      </c>
-      <c r="B61" s="26">
+      <c r="A61" s="25" t="s">
+        <v>129</v>
+      </c>
+      <c r="B61" s="27">
         <f>B42-B54</f>
         <v>359434.25</v>
       </c>
-      <c r="C61" s="26">
+      <c r="C61" s="27">
         <f>IF(C38&gt;0,C42-D54,"")</f>
         <v>349482.46799999994</v>
       </c>
       <c r="F61" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A62" s="24" t="s">
-        <v>130</v>
-      </c>
-      <c r="B62" s="18">
+      <c r="A62" s="25" t="s">
+        <v>131</v>
+      </c>
+      <c r="B62" s="19">
         <f>IFERROR(B61/B22,"")</f>
         <v>5.6603818897637798E-2</v>
       </c>
-      <c r="C62" s="18">
+      <c r="C62" s="19">
         <f>IF(C61="","",IFERROR(C61/B22,""))</f>
         <v>5.5036609133858258E-2</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>132</v>
-      </c>
-      <c r="B63" s="19">
+        <v>133</v>
+      </c>
+      <c r="B63" s="20">
         <f>IFERROR(B22/B38,"")</f>
         <v>11.228504486981123</v>
       </c>
-      <c r="C63" s="19">
+      <c r="C63" s="20">
         <f>IF(C38&gt;0,IFERROR(B22/C38,""),"")</f>
         <v>11.229954089825485</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B64" s="8">
         <f>IFERROR(B61/B7,"")</f>
@@ -2155,7 +2173,7 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="13" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B66" s="14"/>
       <c r="C66" s="14"/>
@@ -2165,7 +2183,7 @@
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B67" s="8">
         <f>IFERROR(B22*Assumptions!$B$20,"")</f>
@@ -2174,7 +2192,7 @@
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B68" s="8">
         <f>IF(C61="","",IFERROR(PV(Assumptions!$B$22/12,Assumptions!$B$23*12,-C61/Assumptions!$B$21/12),""))</f>
@@ -2182,8 +2200,8 @@
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A69" s="24" t="s">
-        <v>137</v>
+      <c r="A69" s="25" t="s">
+        <v>138</v>
       </c>
       <c r="B69" s="8">
         <f>IFERROR(MIN(B67,B68),"")</f>
@@ -2192,7 +2210,7 @@
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B70" s="8">
         <f>IFERROR(B22-B69,"")</f>
@@ -2201,7 +2219,7 @@
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B71" s="8">
         <f>IFERROR(-PMT(Assumptions!$B$22/12,Assumptions!$B$23*12,B69)*12,"")</f>
@@ -2210,16 +2228,16 @@
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>140</v>
-      </c>
-      <c r="B72" s="19">
+        <v>141</v>
+      </c>
+      <c r="B72" s="20">
         <f>IFERROR(C61/B71,"")</f>
         <v>1.2500000000000042</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B73" s="8">
         <f>IFERROR(C61-B71,"")</f>
@@ -2228,21 +2246,21 @@
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>142</v>
-      </c>
-      <c r="B74" s="18">
+        <v>143</v>
+      </c>
+      <c r="B74" s="19">
         <f>IFERROR(B73/B70,"")</f>
         <v>2.7239634488874086E-2</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A3" r:id="rId1" xr:uid="{50A2B422-B5CF-49E6-8BE6-4DB2F0B7B7B0}"/>
+    <hyperlink ref="A3" r:id="rId1" xr:uid="{473D3D7F-B4C1-4234-A58D-59FE728B1101}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" r:id="rId2"/>

</xml_diff>